<commit_message>
test(import): use fictional names in import examples and fixtures
Examples, docstrings, tests and the spreadsheet fixture used names of
real people; they are replaced with obviously fictional ones.
</commit_message>
<xml_diff>
--- a/tests/fixtures/test_import.xlsx
+++ b/tests/fixtures/test_import.xlsx
@@ -462,7 +462,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Novák Jan</t>
+          <t>Příklad Jiří</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -472,7 +472,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>jan.novak@example.cz</t>
+          <t>jiri.priklad@example.cz</t>
         </is>
       </c>
       <c r="D2" t="b">
@@ -540,7 +540,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Svoboda Petr</t>
+          <t>Testovací Patrik</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -550,7 +550,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>petr.svoboda@example.cz</t>
+          <t>patrik.testovaci@example.cz</t>
         </is>
       </c>
       <c r="D5" t="b">
@@ -618,7 +618,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Kratochvíl Tomáš</t>
+          <t>Vzorný Tadeáš</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -628,7 +628,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>tomas.kratochvil@example.cz</t>
+          <t>tadeas.vzorny@example.cz</t>
         </is>
       </c>
       <c r="D8" t="b">
@@ -670,7 +670,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Horáková Marie</t>
+          <t>Ukázková Marta</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -680,7 +680,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>marie.horakova@example.cz</t>
+          <t>marta.ukazkova@example.cz</t>
         </is>
       </c>
       <c r="D10" t="b">
@@ -730,13 +730,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T11"/>
+  <dimension ref="A1:P11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Pro materiál si chodíme předem po domluvě s Míšou či Hankou</t>
+          <t>Pro materiál si chodíme předem po domluvě s Pepou či Mařkou</t>
         </is>
       </c>
     </row>
@@ -856,12 +856,12 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Novák Jan</t>
+          <t>Příklad Jiří</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Svoboda Petr</t>
+          <t>Testovací Patrik</t>
         </is>
       </c>
     </row>
@@ -909,12 +909,12 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Kratochvíl Tomáš</t>
+          <t>Vzorný Tadeáš</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Horáková Marie</t>
+          <t>Ukázková Marta</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -1099,12 +1099,12 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Kratochvíl Tomáš</t>
+          <t>Vzorný Tadeáš</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Novák Jan</t>
+          <t>Příklad Jiří</t>
         </is>
       </c>
     </row>
@@ -1147,12 +1147,12 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Novák Jan</t>
+          <t>Příklad Jiří</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Pokorný Zdeněk</t>
+          <t>Fiktivní Zbyněk</t>
         </is>
       </c>
     </row>
@@ -1195,7 +1195,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Pokorný Zdeněk</t>
+          <t>Fiktivní Zbyněk</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">

</xml_diff>